<commit_message>
feat: add badge generator and update README
- Add new badge generator script with PNG templates and sample data
- Update room plaque generator to improve room number handling and sorting
- Expand README with detailed setup instructions and usage guides for both generators
</commit_message>
<xml_diff>
--- a/gerador_plaquetas/lista_quartos.xlsx
+++ b/gerador_plaquetas/lista_quartos.xlsx
@@ -8,19 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositórios\retiro-manda-teu-fogo\gerador_plaquetas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A341854-C7B7-4D4C-9DB5-52ED4009391A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C428E1-A363-4081-B050-481FC9430D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pessoas" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <definedNames>
+    <definedName name="_Quartos">[1]!Tabela36[Quarto]</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="143">
   <si>
     <t>Nome</t>
   </si>
@@ -515,6 +521,30 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Voluntários - Internos"/>
+      <sheetName val="Voluntários - Externos"/>
+      <sheetName val="Crismandos"/>
+      <sheetName val="Qartos"/>
+      <sheetName val="Equipes- Servos"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2255,7 +2285,7 @@
         <v>142</v>
       </c>
       <c r="D104" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
@@ -2265,8 +2295,8 @@
       <c r="B105" t="s">
         <v>142</v>
       </c>
-      <c r="D105">
-        <v>52</v>
+      <c r="D105" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
@@ -2276,8 +2306,8 @@
       <c r="B106" t="s">
         <v>142</v>
       </c>
-      <c r="D106" t="s">
-        <v>135</v>
+      <c r="D106">
+        <v>52</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
@@ -2288,7 +2318,7 @@
         <v>142</v>
       </c>
       <c r="D107" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
@@ -2310,7 +2340,7 @@
         <v>142</v>
       </c>
       <c r="D109" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
@@ -2320,8 +2350,8 @@
       <c r="B110" t="s">
         <v>142</v>
       </c>
-      <c r="D110">
-        <v>53</v>
+      <c r="D110" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
@@ -2343,7 +2373,7 @@
         <v>142</v>
       </c>
       <c r="D112">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
@@ -2353,8 +2383,8 @@
       <c r="B113" t="s">
         <v>142</v>
       </c>
-      <c r="D113" t="s">
-        <v>138</v>
+      <c r="D113">
+        <v>52</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
@@ -2375,8 +2405,8 @@
       <c r="B115" t="s">
         <v>142</v>
       </c>
-      <c r="D115">
-        <v>53</v>
+      <c r="D115" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
@@ -2386,8 +2416,8 @@
       <c r="B116" t="s">
         <v>142</v>
       </c>
-      <c r="D116" t="s">
-        <v>137</v>
+      <c r="D116">
+        <v>53</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
@@ -2398,7 +2428,7 @@
         <v>142</v>
       </c>
       <c r="D117" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
@@ -2408,8 +2438,8 @@
       <c r="B118" t="s">
         <v>142</v>
       </c>
-      <c r="D118">
-        <v>53</v>
+      <c r="D118" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
@@ -2430,8 +2460,8 @@
       <c r="B120" t="s">
         <v>142</v>
       </c>
-      <c r="D120" t="s">
-        <v>139</v>
+      <c r="D120">
+        <v>53</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
@@ -2442,7 +2472,7 @@
         <v>142</v>
       </c>
       <c r="D121" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
@@ -2453,7 +2483,7 @@
         <v>142</v>
       </c>
       <c r="D122" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
@@ -2464,7 +2494,7 @@
         <v>142</v>
       </c>
       <c r="D123" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
@@ -2473,6 +2503,9 @@
       </c>
       <c r="B124" t="s">
         <v>142</v>
+      </c>
+      <c r="D124" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>